<commit_message>
Update for Fall 2026
</commit_message>
<xml_diff>
--- a/schedule.xlsx
+++ b/schedule.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="31">
   <si>
     <t>Time</t>
   </si>
@@ -94,12 +94,6 @@
     <t>06:30-07:00</t>
   </si>
   <si>
-    <t>07:00-07:30</t>
-  </si>
-  <si>
-    <t>07:30-08:00</t>
-  </si>
-  <si>
     <t>Help Hours</t>
   </si>
   <si>
@@ -109,10 +103,10 @@
     <t>9:30-10:00</t>
   </si>
   <si>
-    <t>STT 4812</t>
-  </si>
-  <si>
-    <t>STT 5811</t>
+    <t>STT 1810</t>
+  </si>
+  <si>
+    <t>STT 4811</t>
   </si>
 </sst>
 </file>
@@ -457,7 +451,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="6" width="15.7109375" style="1" customWidth="1"/>
@@ -485,12 +479,12 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -532,10 +526,10 @@
         <v>11</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>17</v>
@@ -546,10 +540,10 @@
         <v>12</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -560,10 +554,10 @@
         <v>13</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>17</v>
@@ -574,10 +568,10 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -585,24 +579,18 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="D14" s="1" t="s">
         <v>17</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -610,13 +598,13 @@
         <v>18</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -624,13 +612,13 @@
         <v>19</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -638,25 +626,19 @@
         <v>20</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>17</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>28</v>
-      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -665,13 +647,7 @@
       <c r="B19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="D19"/>
-      <c r="E19" s="1" t="s">
-        <v>28</v>
-      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
@@ -697,34 +673,6 @@
       <c r="D21"/>
       <c r="E21"/>
       <c r="F21"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22"/>
-      <c r="E22"/>
-      <c r="F22"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23"/>
-      <c r="E23"/>
-      <c r="F23"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>